<commit_message>
feat: add ecommerce naming fallback for orkli output
</commit_message>
<xml_diff>
--- a/data/input/Datos.xlsx
+++ b/data/input/Datos.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://solerteselen-my.sharepoint.com/personal/jcvega_solerteselen_cat/Documents/Escritorio/jean/Codigo Soler Teselen/script/data/input/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nas18\OneDrive\Escritorio\Soler Teselen\Script\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="13_ncr:1_{36A46A7C-C30A-46B6-90B6-C48F6A49F770}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9620D31B-ED19-45C1-A71B-78C9A4443E5E}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B99E0D38-4080-496F-B425-ABBAFF230EF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9375" yWindow="1170" windowWidth="18855" windowHeight="14310" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="194">
   <si>
     <t>referencia</t>
   </si>
@@ -145,6 +145,468 @@
   </si>
   <si>
     <t>V-05369</t>
+  </si>
+  <si>
+    <t>ORKLI PONT PROVA VALVULA MONOTUB</t>
+  </si>
+  <si>
+    <t>E-19863</t>
+  </si>
+  <si>
+    <t>ORKLI JOC 2 RACCORDS INOX EUROCON 3/4 16X1.8</t>
+  </si>
+  <si>
+    <t>V-04226</t>
+  </si>
+  <si>
+    <t>ORKLI JOC 2 RACCORDS INOX EUROCON 3/4 20X2</t>
+  </si>
+  <si>
+    <t>V-04229</t>
+  </si>
+  <si>
+    <t>ORKLI RACOR TERMOSTATIC PER COLECTORS MODULARS</t>
+  </si>
+  <si>
+    <t>E-25092</t>
+  </si>
+  <si>
+    <t>ORKLI CAUDALIMETRO GRUPO HIDRAULICO 74400</t>
+  </si>
+  <si>
+    <t>V-03816</t>
+  </si>
+  <si>
+    <t>ORKLI ARMARI METAL·LIC EMPOTRAR  840X510X90/130</t>
+  </si>
+  <si>
+    <t>1008090</t>
+  </si>
+  <si>
+    <t>ORKLI ARMARI PLASTIC 335X275X88</t>
+  </si>
+  <si>
+    <t>E-18620</t>
+  </si>
+  <si>
+    <t>ORKLI ARMARI PLASTIC 415X275X88</t>
+  </si>
+  <si>
+    <t>E-18621</t>
+  </si>
+  <si>
+    <t>ORKLI ARMARI PLASTIC 515X275X88</t>
+  </si>
+  <si>
+    <t>E-18622</t>
+  </si>
+  <si>
+    <t>ORKLI CAPÇAL TERMOELECTRIC M30X1,5 NC 230V</t>
+  </si>
+  <si>
+    <t>CT410800</t>
+  </si>
+  <si>
+    <t>ORKLI CAPÇAL TERMOELECTRIC M30X1,5 NC 230V MICRO</t>
+  </si>
+  <si>
+    <t>V-05001</t>
+  </si>
+  <si>
+    <t>ORKLI COL·LECTOR INOX MUNTAT 3/4 COMPLET 5 SORTIDES</t>
+  </si>
+  <si>
+    <t>SM1005S</t>
+  </si>
+  <si>
+    <t>ORKLI COL·LECTOR-VALVULA M-F 3/4-M24X1,5  2 SORTIDES</t>
+  </si>
+  <si>
+    <t>CM35100</t>
+  </si>
+  <si>
+    <t>ORKLI COL·LECTOR-VALVULA M-F 3/4-M24X1,5  3 SORTIDES</t>
+  </si>
+  <si>
+    <t>CM35101</t>
+  </si>
+  <si>
+    <t>ORKLI COL·LECTOR-VALVULA M-F 3/4-M24X1,5  4 SORTIDES</t>
+  </si>
+  <si>
+    <t>CM35102</t>
+  </si>
+  <si>
+    <t>ORKLI COL·LECTOR-VALVULA M-F 1"-M24X1,5  3 SORTIDES</t>
+  </si>
+  <si>
+    <t>CM35104</t>
+  </si>
+  <si>
+    <t>ORKLI COL·LECTOR-VALVULA M-F 1"-M24X1,5  4 SORTIDES</t>
+  </si>
+  <si>
+    <t>CM35105</t>
+  </si>
+  <si>
+    <t>ORKLI RACCORD ADAPTADOR CAPÇAL M28X1</t>
+  </si>
+  <si>
+    <t>V-02214</t>
+  </si>
+  <si>
+    <t>ORKLI RACCORD ADAPTADOR CAPÇAL M30X1,5</t>
+  </si>
+  <si>
+    <t>V-02070</t>
+  </si>
+  <si>
+    <t>ORKLI MODUL COL.LECTOR RETORN 2V 1" CS2200</t>
+  </si>
+  <si>
+    <t>CS2200</t>
+  </si>
+  <si>
+    <t>ORKLI MODUL COL.LECTOR RETORN 3V 1" CS3200</t>
+  </si>
+  <si>
+    <t>CS3200</t>
+  </si>
+  <si>
+    <t>ORKLI MONTURA COL-LECTOR LLAUTO E-24881</t>
+  </si>
+  <si>
+    <t>E-24881</t>
+  </si>
+  <si>
+    <t>ORKLI CRONOTERMOSTAT AMBIENT ON-OF RA300</t>
+  </si>
+  <si>
+    <t>RA300</t>
+  </si>
+  <si>
+    <t>ORKLI TERMOSTAT AMBIENT DIGITAL ESTIU-HIV. RA210</t>
+  </si>
+  <si>
+    <t>RA210</t>
+  </si>
+  <si>
+    <t>ORKLI TERMOSTAT AMBIENT DIGITAL ON-OFF RA200</t>
+  </si>
+  <si>
+    <t>RA200</t>
+  </si>
+  <si>
+    <t>ORKLI TERMOSTAT AMBIENT MECANIC ESTIU-HIV. RA110</t>
+  </si>
+  <si>
+    <t>RA110</t>
+  </si>
+  <si>
+    <t>ORKLI TERMOSTAT AMBIENT MECANIC ON-OF RA100</t>
+  </si>
+  <si>
+    <t>RA100</t>
+  </si>
+  <si>
+    <t>ORKLI VALVULA ZONA CLASICA MICRO 2 VIES  3/4</t>
+  </si>
+  <si>
+    <t>30223200</t>
+  </si>
+  <si>
+    <t>ORKLI VALVULA ZONA CLASICA MICRO 2 VIES 1"</t>
+  </si>
+  <si>
+    <t>30323200</t>
+  </si>
+  <si>
+    <t>ORKLI VALVULA ZONA CLASICA MICRO 3 VIES  3/4</t>
+  </si>
+  <si>
+    <t>40223200</t>
+  </si>
+  <si>
+    <t>ORKLI VALVULA ZONA CLASICA MICRO 3 VIES 1"</t>
+  </si>
+  <si>
+    <t>40323200</t>
+  </si>
+  <si>
+    <t>ORKLI VALVULA ZONA CLASICA S/MICRO 2 VIES  1/2</t>
+  </si>
+  <si>
+    <t>30113200</t>
+  </si>
+  <si>
+    <t>ORKLI VALVULA ZONA CLASICA S/MICRO 2 VIES  3/4</t>
+  </si>
+  <si>
+    <t>30213200</t>
+  </si>
+  <si>
+    <t>ORKLI VALVULA ZONA CLASICA S/MICRO 2 VIES 1"</t>
+  </si>
+  <si>
+    <t>30313200</t>
+  </si>
+  <si>
+    <t>ORKLI VALVULA ZONA CLASICA S/MICRO 3VIES  1/2</t>
+  </si>
+  <si>
+    <t>40113200</t>
+  </si>
+  <si>
+    <t>ORKLI VALVULA ZONA CLASICA S/MICRO 3VIES  3/4</t>
+  </si>
+  <si>
+    <t>40213200</t>
+  </si>
+  <si>
+    <t>ORKLI VALVULA ZONA CLASICA S/MICRO 3 VIES 1"</t>
+  </si>
+  <si>
+    <t>40313200</t>
+  </si>
+  <si>
+    <t>ORKLI TUBERIA PEX-A ROTLLE EVOH 16X1.8</t>
+  </si>
+  <si>
+    <t>SRTBA16-200</t>
+  </si>
+  <si>
+    <t>ORKLI ACTUADOR VALVULA ZONA NEW AMB MICRO 240V</t>
+  </si>
+  <si>
+    <t>50024200</t>
+  </si>
+  <si>
+    <t>ORKLI ACTUADOR VALVULA ZONA NEW S/MICRO 240V</t>
+  </si>
+  <si>
+    <t>50014200</t>
+  </si>
+  <si>
+    <t>ORKLI COS VALVULA ZONA NEW  2 VIES  1/2</t>
+  </si>
+  <si>
+    <t>39104000</t>
+  </si>
+  <si>
+    <t>ORKLI COS VALVULA ZONA NEW  2 VIES  3/4</t>
+  </si>
+  <si>
+    <t>39204000</t>
+  </si>
+  <si>
+    <t>ORKLI COS VALVULA ZONA NEW  2 VIES   1"</t>
+  </si>
+  <si>
+    <t>39304000</t>
+  </si>
+  <si>
+    <t>ORKLI COS VALVULA ZONA NEW  3 VIES  1/2</t>
+  </si>
+  <si>
+    <t>49104000</t>
+  </si>
+  <si>
+    <t>ORKLI COS VALVULA ZONA NEW  3 VIES  3/4</t>
+  </si>
+  <si>
+    <t>49204000</t>
+  </si>
+  <si>
+    <t>ORKLI COS VALVULA ZONA NEW  3 VIES   1"</t>
+  </si>
+  <si>
+    <t>49304000</t>
+  </si>
+  <si>
+    <t>ORKLI GRUP SEGURETAT STANDARD RECTE 7K. 3/4</t>
+  </si>
+  <si>
+    <t>GS1110000</t>
+  </si>
+  <si>
+    <t>ORKLI VALVULA CALDERA CONNEXIO CALEFACCIO 3/4</t>
+  </si>
+  <si>
+    <t>91399-00</t>
+  </si>
+  <si>
+    <t>ORKLI VALVULA SEGURETAT VS 1/2-3K</t>
+  </si>
+  <si>
+    <t>17003-00</t>
+  </si>
+  <si>
+    <t>ORKLI VALVULA SEGURETAT VS 1/2-3K AMB TOMA MAN.</t>
+  </si>
+  <si>
+    <t>17004-00</t>
+  </si>
+  <si>
+    <t>ORKLI VALVULA SEGURETAT VS 1/2-7K</t>
+  </si>
+  <si>
+    <t>17011-01</t>
+  </si>
+  <si>
+    <t>ORKLI VALVULA SEGURETAT VSM 1/2-3K MANOMETRE</t>
+  </si>
+  <si>
+    <t>17004-01</t>
+  </si>
+  <si>
+    <t>ORKLI CAPÇAL TERMOSTATIC HARMONY LX LIQUID</t>
+  </si>
+  <si>
+    <t>60010</t>
+  </si>
+  <si>
+    <t>ORKLI DETENTOR RADIADOR  3/8X12-20 ESC.</t>
+  </si>
+  <si>
+    <t>87210</t>
+  </si>
+  <si>
+    <t>ORKLI DETENTOR RADIADOR 1/2X12-20 ESC.</t>
+  </si>
+  <si>
+    <t>1220</t>
+  </si>
+  <si>
+    <t>ORKLI DETENTOR RADIADOR ROSCAR  3/8 ESC.</t>
+  </si>
+  <si>
+    <t>1015</t>
+  </si>
+  <si>
+    <t>ORKLI DETENTOR RADIADOR ROSCAR 1/2 ESC.</t>
+  </si>
+  <si>
+    <t>1025</t>
+  </si>
+  <si>
+    <t>ORKLI DETENTOR RADIADOR SOLDAR 15X1/2 ESC.</t>
+  </si>
+  <si>
+    <t>1425</t>
+  </si>
+  <si>
+    <t>ORKLI VALVULA BITUB TERMT. 1/2X12-20 52490</t>
+  </si>
+  <si>
+    <t>52490</t>
+  </si>
+  <si>
+    <t>ORKLI VALVULA BITUB TERMT. 1/2X12-20 52720</t>
+  </si>
+  <si>
+    <t>52720</t>
+  </si>
+  <si>
+    <t>ORKLI VALVULA MONOTUB NIQ. 1/2 S/REG.</t>
+  </si>
+  <si>
+    <t>1816</t>
+  </si>
+  <si>
+    <t>ORKLI VALVULA MONOTUB NIQ. 1/2-18 D/REG.</t>
+  </si>
+  <si>
+    <t>1866</t>
+  </si>
+  <si>
+    <t>ORKLI VALVULA MONOTUB NIQ. 1/2-18 S/REG.</t>
+  </si>
+  <si>
+    <t>1817</t>
+  </si>
+  <si>
+    <t>ORKLI VALVULA MONOTUB TERMT. 1/2X12-20 52390</t>
+  </si>
+  <si>
+    <t>52390</t>
+  </si>
+  <si>
+    <t>ORKLI VALVULA MONOTUB TERMT. 1/2X12-20 52710</t>
+  </si>
+  <si>
+    <t>52710</t>
+  </si>
+  <si>
+    <t>ORKLI VALVULA MONOTUB TERMT. D 1/2X12-20 52310</t>
+  </si>
+  <si>
+    <t>52310</t>
+  </si>
+  <si>
+    <t>ORKLI VALVULA MONOTUB TERMT. E 1/2X12-20 52110</t>
+  </si>
+  <si>
+    <t>52110</t>
+  </si>
+  <si>
+    <t>ORKLI VALVULA RADIADOR 3/8X12-20 ESC.</t>
+  </si>
+  <si>
+    <t>81210</t>
+  </si>
+  <si>
+    <t>ORKLI VALVULA RADIADOR 1/2X12-20 ESC.</t>
+  </si>
+  <si>
+    <t>82210</t>
+  </si>
+  <si>
+    <t>ORKLI VALVULA RADIADOR ROSCAR  3/8 ESC.</t>
+  </si>
+  <si>
+    <t>1115</t>
+  </si>
+  <si>
+    <t>ORKLI VALVULA RADIADOR ROSCAR 1/2 ESC.</t>
+  </si>
+  <si>
+    <t>1125</t>
+  </si>
+  <si>
+    <t>ORKLI VALVULA RADIADOR SOLDAR 15X1/2 ESC.</t>
+  </si>
+  <si>
+    <t>1325</t>
+  </si>
+  <si>
+    <t>ORKLI VALVULA RADIADOR TERMT. ROSCAR  3/8 ESC.</t>
+  </si>
+  <si>
+    <t>67150</t>
+  </si>
+  <si>
+    <t>ORKLI VALVULA RADIADOR TERMT. ROSCAR 1/2 ESC.</t>
+  </si>
+  <si>
+    <t>67450</t>
+  </si>
+  <si>
+    <t>ORKLI VALVULA RADIADOR TERMT. SOLDAR 15X1/2 ESC.</t>
+  </si>
+  <si>
+    <t>67401</t>
+  </si>
+  <si>
+    <t>ORKLI VALVULA RADIADOR TERMT. M24X1,5 - 1/2 ESC.</t>
+  </si>
+  <si>
+    <t>67490</t>
+  </si>
+  <si>
+    <t>ORKLI VALVULA RADIADOR TERMT. M24X1,5 - 1/2 ESC. INVERTIDA</t>
+  </si>
+  <si>
+    <t>67690</t>
   </si>
 </sst>
 </file>
@@ -462,7 +924,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B99"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="51.85546875" bestFit="1" customWidth="1"/>
@@ -495,138 +957,770 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B9" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B11" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B12" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B13" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B14" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B15" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B16" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="B17" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B18" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B19" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>34</v>
+      </c>
+      <c r="B20" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>36</v>
+      </c>
+      <c r="B21" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>38</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B22" t="s">
         <v>39</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>40</v>
+      </c>
+      <c r="B23" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>42</v>
+      </c>
+      <c r="B24" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>44</v>
+      </c>
+      <c r="B25" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>48</v>
+      </c>
+      <c r="B27" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>50</v>
+      </c>
+      <c r="B28" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>52</v>
+      </c>
+      <c r="B29" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>54</v>
+      </c>
+      <c r="B30" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>56</v>
+      </c>
+      <c r="B31" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>58</v>
+      </c>
+      <c r="B32" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>60</v>
+      </c>
+      <c r="B33" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>62</v>
+      </c>
+      <c r="B34" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>64</v>
+      </c>
+      <c r="B35" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>66</v>
+      </c>
+      <c r="B36" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>68</v>
+      </c>
+      <c r="B37" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>70</v>
+      </c>
+      <c r="B38" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>72</v>
+      </c>
+      <c r="B39" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>74</v>
+      </c>
+      <c r="B40" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>76</v>
+      </c>
+      <c r="B41" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>78</v>
+      </c>
+      <c r="B42" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>80</v>
+      </c>
+      <c r="B43" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>82</v>
+      </c>
+      <c r="B44" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>84</v>
+      </c>
+      <c r="B45" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>86</v>
+      </c>
+      <c r="B46" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>88</v>
+      </c>
+      <c r="B47" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>90</v>
+      </c>
+      <c r="B48" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>92</v>
+      </c>
+      <c r="B49" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>94</v>
+      </c>
+      <c r="B50" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>96</v>
+      </c>
+      <c r="B51" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>98</v>
+      </c>
+      <c r="B52" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>100</v>
+      </c>
+      <c r="B53" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>102</v>
+      </c>
+      <c r="B54" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>104</v>
+      </c>
+      <c r="B55" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>106</v>
+      </c>
+      <c r="B56" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>108</v>
+      </c>
+      <c r="B57" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>110</v>
+      </c>
+      <c r="B58" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>112</v>
+      </c>
+      <c r="B59" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>114</v>
+      </c>
+      <c r="B60" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>116</v>
+      </c>
+      <c r="B61" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>118</v>
+      </c>
+      <c r="B62" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>120</v>
+      </c>
+      <c r="B63" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>122</v>
+      </c>
+      <c r="B64" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>124</v>
+      </c>
+      <c r="B65" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>126</v>
+      </c>
+      <c r="B66" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>128</v>
+      </c>
+      <c r="B67" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>130</v>
+      </c>
+      <c r="B68" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>132</v>
+      </c>
+      <c r="B69" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>134</v>
+      </c>
+      <c r="B70" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>136</v>
+      </c>
+      <c r="B71" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>138</v>
+      </c>
+      <c r="B72" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>140</v>
+      </c>
+      <c r="B73" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>142</v>
+      </c>
+      <c r="B74" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>144</v>
+      </c>
+      <c r="B75" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>146</v>
+      </c>
+      <c r="B76" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>148</v>
+      </c>
+      <c r="B77" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>150</v>
+      </c>
+      <c r="B78" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>152</v>
+      </c>
+      <c r="B79" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>154</v>
+      </c>
+      <c r="B80" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>156</v>
+      </c>
+      <c r="B81" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>158</v>
+      </c>
+      <c r="B82" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>160</v>
+      </c>
+      <c r="B83" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>162</v>
+      </c>
+      <c r="B84" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>164</v>
+      </c>
+      <c r="B85" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>166</v>
+      </c>
+      <c r="B86" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>168</v>
+      </c>
+      <c r="B87" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>170</v>
+      </c>
+      <c r="B88" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>172</v>
+      </c>
+      <c r="B89" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>174</v>
+      </c>
+      <c r="B90" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>176</v>
+      </c>
+      <c r="B91" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>178</v>
+      </c>
+      <c r="B92" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>180</v>
+      </c>
+      <c r="B93" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>182</v>
+      </c>
+      <c r="B94" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>184</v>
+      </c>
+      <c r="B95" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>186</v>
+      </c>
+      <c r="B96" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>188</v>
+      </c>
+      <c r="B97" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>190</v>
+      </c>
+      <c r="B98" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>192</v>
+      </c>
+      <c r="B99" t="s">
+        <v>193</v>
       </c>
     </row>
   </sheetData>

</xml_diff>